<commit_message>
Ajout de fichier result
</commit_message>
<xml_diff>
--- a/FichierControleFluxCoteUnix/rapport/10082026_FOURNISSEUR_VFF.xlsx
+++ b/FichierControleFluxCoteUnix/rapport/10082026_FOURNISSEUR_VFF.xlsx
@@ -11,12 +11,28 @@
     <sheet name="Factures a 0" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Synthese Oracle" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Detail Oracle" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Synthese 100826_114541" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Factures a 0 100826_114541" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Synthese Oracle 100826_114541" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Detail Oracle 100826_114541" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Synthese 100826_114631" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Factures a 0 100826_114631" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Synthese Oracle 100826_114631" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Detail Oracle 100826_114631" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Synthese'!$A$6:$F$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Factures a 0'!$A$4:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Synthese Oracle'!$A$4:$I$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Detail Oracle'!$A$4:$G$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Synthese 100826_114541'!$A$6:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Factures a 0 100826_114541'!$A$4:$D$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Synthese Oracle 100826_114541'!$A$4:$I$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Detail Oracle 100826_114541'!$A$4:$G$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Synthese 100826_114631'!$A$6:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Factures a 0 100826_114631'!$A$4:$D$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Synthese Oracle 100826_114631'!$A$4:$I$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Detail Oracle 100826_114631'!$A$4:$G$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -623,6 +639,1098 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FACTURES A MONTANT ZERO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fichier source</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>VHC03_SRC_FACTURESFOURNISSEURS_100826_114631.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Folio</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>N° facture</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Compte</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Date piece</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Aucune facture a montant 0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:D5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CONTROLE FAC02 FOURNISSEURS - SYNTHESE ORACLE PAR FOLIO</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
+      <c r="E1" s="11" t="n"/>
+      <c r="F1" s="11" t="n"/>
+      <c r="G1" s="11" t="n"/>
+      <c r="H1" s="11" t="n"/>
+      <c r="I1" s="11" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Fichier : VHC03_SRC_FACTURESFOURNISSEURS_100826_114631  |  Execution : 26/08/2026 14:44:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Folio</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Fichier</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Nb Factures Fichier</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Montant Fichier</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Nb Factures Oracle</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Montant Oracle</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Nb Factures Interface</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Montant Interface</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>VHC03_SRC_FACTURESFOURNISSEURS_100826_114631</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>5633.38</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>ECART</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:I5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CONTROLE FAC02 FOURNISSEURS - DETAIL FACTURE PAR FACTURE</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
+      <c r="E1" s="11" t="n"/>
+      <c r="F1" s="11" t="n"/>
+      <c r="G1" s="11" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Fichier : VHC03_SRC_FACTURESFOURNISSEURS_100826_114631  |  Execution : 26/08/2026 14:44:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Folio</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Numero Piece</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Date Piece</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Montant Fichier</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Montant Oracle</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Montant Interface</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>FR1181216</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>31/05/2025</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>808.73</v>
+      </c>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>FR1153339</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>31/10/2024</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>1692.2</v>
+      </c>
+      <c r="E6" s="15" t="n"/>
+      <c r="F6" s="15" t="n"/>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>FR1196986</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>31/10/2025</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>94.36</v>
+      </c>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>FR1196987</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>31/10/2025</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="n">
+        <v>26.96</v>
+      </c>
+      <c r="E8" s="15" t="n"/>
+      <c r="F8" s="15" t="n"/>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>FR1196988</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>31/10/2025</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>53.92</v>
+      </c>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>FR1196989</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>31/10/2025</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>53.92</v>
+      </c>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>FR1196990</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>31/10/2025</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>13.48</v>
+      </c>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>FR1196991</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>31/10/2025</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>13.48</v>
+      </c>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>FR1197910</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>31/10/2025</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>40.44</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>40.44</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>40.44</v>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>INTEGREE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>FR1225990</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>30/04/2026</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>INTEGREE</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>FR1225991</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>30/04/2026</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>INTEGREE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>FR1221715</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>31/03/2026</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>INTEGREE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>FR1221716</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>31/03/2026</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>INTEGREE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>FR1217484</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>28/02/2026</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>FR1217485</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>28/02/2026</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>FR1201975</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>30/11/2025</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>26.96</v>
+      </c>
+      <c r="E20" s="15" t="n"/>
+      <c r="F20" s="15" t="n"/>
+      <c r="G20" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>FR1201977</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>30/11/2025</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>53.92</v>
+      </c>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>FR1201976</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>30/11/2025</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="n">
+        <v>53.92</v>
+      </c>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="15" t="n"/>
+      <c r="G22" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>FR1201979</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>30/11/2025</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>53.91</v>
+      </c>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>FR1201974</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>30/11/2025</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="n">
+        <v>94.36</v>
+      </c>
+      <c r="E24" s="15" t="n"/>
+      <c r="F24" s="15" t="n"/>
+      <c r="G24" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>FR1201978</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>30/11/2025</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>13.48</v>
+      </c>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>FR1181210</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>31/05/2025</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="n">
+        <v>134.79</v>
+      </c>
+      <c r="E26" s="15" t="n"/>
+      <c r="F26" s="15" t="n"/>
+      <c r="G26" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>FR1137566</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>31/07/2024</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>236.15</v>
+      </c>
+      <c r="E27" s="7" t="n"/>
+      <c r="F27" s="7" t="n"/>
+      <c r="G27" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>FR1141749</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>31/07/2024</t>
+        </is>
+      </c>
+      <c r="D28" s="15" t="n">
+        <v>1206.75</v>
+      </c>
+      <c r="E28" s="15" t="n"/>
+      <c r="F28" s="15" t="n"/>
+      <c r="G28" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>FR1137567</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>31/07/2024</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>314.82</v>
+      </c>
+      <c r="E29" s="7" t="n"/>
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>FR1137564</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>31/07/2024</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="E30" s="15" t="n"/>
+      <c r="F30" s="15" t="n"/>
+      <c r="G30" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>FR1137565</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>31/07/2024</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>367.29</v>
+      </c>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="n"/>
+      <c r="G31" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>FR1137569</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>31/07/2024</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>118.08</v>
+      </c>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" s="15" t="n"/>
+      <c r="G32" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>FR1137568</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>31/07/2024</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>13.12</v>
+      </c>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="7" t="n"/>
+      <c r="G33" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:G33"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -721,14 +1829,6 @@
           <t>CONTROLE FAC02 FOURNISSEURS - SYNTHESE ORACLE PAR FOLIO</t>
         </is>
       </c>
-      <c r="B1" s="11" t="n"/>
-      <c r="C1" s="11" t="n"/>
-      <c r="D1" s="11" t="n"/>
-      <c r="E1" s="11" t="n"/>
-      <c r="F1" s="11" t="n"/>
-      <c r="G1" s="11" t="n"/>
-      <c r="H1" s="11" t="n"/>
-      <c r="I1" s="11" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -852,12 +1952,6 @@
           <t>CONTROLE FAC02 FOURNISSEURS - DETAIL FACTURE PAR FACTURE</t>
         </is>
       </c>
-      <c r="B1" s="11" t="n"/>
-      <c r="C1" s="11" t="n"/>
-      <c r="D1" s="11" t="n"/>
-      <c r="E1" s="11" t="n"/>
-      <c r="F1" s="11" t="n"/>
-      <c r="G1" s="11" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1713,4 +2807,588 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CONTROLE FLUX FAC02 - FACTURES FOURNISSEURS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fichier SRC</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>VHC03_SRC_FACTURESFOURNISSEURS_100826_114541.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Fichier CTL</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>VHC03_CTL_FACTURESFOURNISSEURS_100826_114541.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Resultat</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>RAPPROCHEMENT OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Folio</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Nb factures SRC</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Montant SRC</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Nb factures CTL</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Montant CTL</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>672.72</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>672.72</v>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>672.72</v>
+      </c>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="9" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:F7"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FACTURES A MONTANT ZERO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fichier source</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>VHC03_SRC_FACTURESFOURNISSEURS_100826_114541.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Folio</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>N° facture</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Compte</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Date piece</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Aucune facture a montant 0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:D5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CONTROLE FAC02 FOURNISSEURS - SYNTHESE ORACLE PAR FOLIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Fichier : VHC03_SRC_FACTURESFOURNISSEURS_100826_114541  |  Execution : 26/08/2026 14:44:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Folio</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Fichier</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Nb Factures Fichier</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Montant Fichier</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Nb Factures Oracle</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Montant Oracle</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Nb Factures Interface</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Montant Interface</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>VHC03_SRC_FACTURESFOURNISSEURS_100826_114541</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>672.72</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:I5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CONTROLE FAC02 FOURNISSEURS - DETAIL FACTURE PAR FACTURE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Fichier : VHC03_SRC_FACTURESFOURNISSEURS_100826_114541  |  Execution : 26/08/2026 14:44:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Folio</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Numero Piece</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Date Piece</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Montant Fichier</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Montant Oracle</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Montant Interface</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>24/12/2025</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>24/12/2025</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>672.72</v>
+      </c>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>ABSENTE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:G5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CONTROLE FLUX FAC02 - FACTURES FOURNISSEURS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fichier SRC</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>VHC03_SRC_FACTURESFOURNISSEURS_100826_114631.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Fichier CTL</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>VHC03_CTL_FACTURESFOURNISSEURS_100826_114631.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Resultat</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>RAPPROCHEMENT OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Folio</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Nb factures SRC</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Montant SRC</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Nb factures CTL</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Montant CTL</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>5633.38</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>5633.38</v>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>5633.38</v>
+      </c>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="9" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A6:F7"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>